<commit_message>
docs: document custom player draw layers and refresh API catalog
</commit_message>
<xml_diff>
--- a/docs/referencia/metodos.xlsx
+++ b/docs/referencia/metodos.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Índice" sheetId="1" r:id="Re64c2067295546fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Métodos" sheetId="2" r:id="Rf2d3f4f78cd141c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Índice" sheetId="1" r:id="R5e16950c57f341e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Métodos" sheetId="2" r:id="R9b76389d2d924fa5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -165,8 +165,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MetodosPublicos" displayName="MetodosPublicos" ref="A6:K1077" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:K1077"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MetodosPublicos" displayName="MetodosPublicos" ref="A6:K1084" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:K1084"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Classe"/>
     <x:tableColumn id="2" name="Método"/>
@@ -407,7 +407,7 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>64 classes. 1061 registros declarados. 10 métodos não implementados.</x:v>
+        <x:v>64 classes. 1068 registros declarados. 10 métodos não implementados.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1337,13 +1337,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="C59" s="6" t="n">
-        <x:v>4</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D59" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E59" s="6" t="n">
-        <x:v>4</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="22" customHeight="1">
@@ -1536,7 +1536,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1290bb2509b549ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff75a8d7ba2c4c62"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35345,7 +35345,7 @@
       </x:c>
       <x:c r="J1008" s="16" t="str"/>
       <x:c r="K1008" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L5</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L11</x:v>
       </x:c>
     </x:row>
     <x:row r="1009" ht="21.75" customHeight="1">
@@ -35378,7 +35378,7 @@
       </x:c>
       <x:c r="J1009" s="16" t="str"/>
       <x:c r="K1009" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L4</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L10</x:v>
       </x:c>
     </x:row>
     <x:row r="1010" ht="34.5" customHeight="1">
@@ -35392,7 +35392,7 @@
         <x:v>Construtor</x:v>
       </x:c>
       <x:c r="D1010" s="16" t="str">
-        <x:v>constructor(name, method)</x:v>
+        <x:v>constructor(name, method = null)</x:v>
       </x:c>
       <x:c r="E1010" s="16" t="str">
         <x:v>PlayerDrawLayer</x:v>
@@ -35407,25 +35407,25 @@
         <x:v>instância</x:v>
       </x:c>
       <x:c r="I1010" s="16" t="str">
-        <x:v>Consulte a implementação na fonte. Descritor de uma camada nativa. Hide e posições BeforeParent/AfterParent atuam no desenho atual. Não registra um novo renderer.</x:v>
+        <x:v>Consulte a implementação na fonte. Base de camadas personalizadas e descritor das nativas. Classes exportadas são registradas automaticamente; o nome padrão é o nome da classe.</x:v>
       </x:c>
       <x:c r="J1010" s="16" t="str"/>
       <x:c r="K1010" s="16" t="str">
         <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L2</x:v>
       </x:c>
     </x:row>
-    <x:row r="1011" ht="21.75" customHeight="1">
+    <x:row r="1011" ht="34.5" customHeight="1">
       <x:c r="A1011" s="16" t="str">
         <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="B1011" s="16" t="str">
-        <x:v>Hide</x:v>
+        <x:v>Draw</x:v>
       </x:c>
       <x:c r="C1011" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1011" s="16" t="str">
-        <x:v>Hide()</x:v>
+        <x:v>Draw(drawInfo)</x:v>
       </x:c>
       <x:c r="E1011" s="16" t="str">
         <x:v>PlayerDrawLayer</x:v>
@@ -35437,31 +35437,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1011" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>undefined</x:v>
       </x:c>
       <x:c r="I1011" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>A implementação base não executa ações. Obrigatório. Adicione DrawData com ModPlayer.AddDrawData(drawInfo, drawData). Executado junto do pai, antes das transformações e da renderização nativas.</x:v>
       </x:c>
       <x:c r="J1011" s="16" t="str"/>
       <x:c r="K1011" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1012" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1012" ht="34.5" customHeight="1">
       <x:c r="A1012" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="B1012" s="16" t="str">
-        <x:v>AllowPrefix</x:v>
+        <x:v>FullName</x:v>
       </x:c>
       <x:c r="C1012" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Getter</x:v>
       </x:c>
       <x:c r="D1012" s="16" t="str">
-        <x:v>AllowPrefix(item, pre)</x:v>
+        <x:v>get FullName</x:v>
       </x:c>
       <x:c r="E1012" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="F1012" s="16" t="str">
         <x:v>Não</x:v>
@@ -35470,31 +35470,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1012" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>this.Mod ? this.Mod.uuid + '/' + this.Name : this.Name</x:v>
       </x:c>
       <x:c r="I1012" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>Consulte a implementação na fonte. Nome qualificado como uuid-do-mod/nome-da-camada.</x:v>
       </x:c>
       <x:c r="J1012" s="16" t="str"/>
       <x:c r="K1012" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L122</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1013" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1013" ht="34.5" customHeight="1">
       <x:c r="A1013" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="B1013" s="16" t="str">
-        <x:v>Categories</x:v>
+        <x:v>GetDefaultPosition</x:v>
       </x:c>
       <x:c r="C1013" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1013" s="16" t="str">
-        <x:v>Categories(item)</x:v>
+        <x:v>GetDefaultPosition()</x:v>
       </x:c>
       <x:c r="E1013" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="F1013" s="16" t="str">
         <x:v>Não</x:v>
@@ -35506,28 +35506,28 @@
         <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1013" s="16" t="str">
-        <x:v>As categorias do item; os prefixos do jogo de uma categoria.</x:v>
+        <x:v>Consulte a implementação na fonte. Obrigatório. Retorne BeforeParent ou AfterParent com descritor nativo, classe registrada, instância ou nome completo. Posições padrão ficam em cache.</x:v>
       </x:c>
       <x:c r="J1013" s="16" t="str"/>
       <x:c r="K1013" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L83</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1014" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1014" ht="34.5" customHeight="1">
       <x:c r="A1014" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="B1014" s="16" t="str">
-        <x:v>GetPrefix</x:v>
+        <x:v>GetDefaultVisibility</x:v>
       </x:c>
       <x:c r="C1014" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1014" s="16" t="str">
-        <x:v>GetPrefix(type)</x:v>
+        <x:v>GetDefaultVisibility(drawInfo)</x:v>
       </x:c>
       <x:c r="E1014" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="F1014" s="16" t="str">
         <x:v>Não</x:v>
@@ -35536,31 +35536,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1014" s="16" t="str">
-        <x:v>PrefixLoader.ByType.get(type)</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="I1014" s="16" t="str">
-        <x:v>O ModPrefix, ou undefined (prefixo do jogo).</x:v>
+        <x:v>Consulte a implementação na fonte. Consultado em cada desenho e para cada jogador. false oculta a camada e seus filhos. Verifique drawInfo.shadow para excluir pós-imagens.</x:v>
       </x:c>
       <x:c r="J1014" s="16" t="str"/>
       <x:c r="K1014" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1015" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1015" ht="34.5" customHeight="1">
       <x:c r="A1015" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="B1015" s="16" t="str">
-        <x:v>GetPrefixesInCategory</x:v>
+        <x:v>Hide</x:v>
       </x:c>
       <x:c r="C1015" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1015" s="16" t="str">
-        <x:v>GetPrefixesInCategory(category)</x:v>
+        <x:v>Hide()</x:v>
       </x:c>
       <x:c r="E1015" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="F1015" s="16" t="str">
         <x:v>Não</x:v>
@@ -35569,31 +35569,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1015" s="16" t="str">
-        <x:v>PrefixLoader.#byCategory.get(category) || []</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1015" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>Consulte a implementação na fonte. Oculta a camada e seus filhos no desenho atual. O estado é restaurado ao terminar, inclusive em chamadas aninhadas.</x:v>
       </x:c>
       <x:c r="J1015" s="16" t="str"/>
       <x:c r="K1015" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L28</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1016" ht="47.25" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1016" ht="34.5" customHeight="1">
       <x:c r="A1016" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="B1016" s="16" t="str">
-        <x:v>IsWeaponSubCategory</x:v>
+        <x:v>register</x:v>
       </x:c>
       <x:c r="C1016" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1016" s="16" t="str">
-        <x:v>IsWeaponSubCategory(category)</x:v>
+        <x:v>register(cls)</x:v>
       </x:c>
       <x:c r="E1016" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="F1016" s="16" t="str">
         <x:v>Não</x:v>
@@ -35602,31 +35602,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1016" s="16" t="str">
-        <x:v>category === PrefixCategory.Melee || category === PrefixCategory.Ranged || category === PrefixCategory.Magic</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1016" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>Registra. Registro manual para classes com Autoload=false ou criadas em execução. Valida Draw e GetDefaultPosition, rejeita duplicatas e cria o template de ModContent.GetInstance.</x:v>
       </x:c>
       <x:c r="J1016" s="16" t="str"/>
       <x:c r="K1016" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L30</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1017" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1017" ht="34.5" customHeight="1">
       <x:c r="A1017" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="B1017" s="16" t="str">
-        <x:v>PrefixCount</x:v>
+        <x:v>SetStaticDefaults</x:v>
       </x:c>
       <x:c r="C1017" s="16" t="str">
-        <x:v>Getter estático</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1017" s="16" t="str">
-        <x:v>get PrefixCount</x:v>
+        <x:v>SetStaticDefaults()</x:v>
       </x:c>
       <x:c r="E1017" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="F1017" s="16" t="str">
         <x:v>Não</x:v>
@@ -35635,31 +35635,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1017" s="16" t="str">
-        <x:v>PrefixLoader.VanillaCount + PrefixLoader.ByType.size</x:v>
+        <x:v>undefined</x:v>
       </x:c>
       <x:c r="I1017" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>A implementação base não executa ações. Uma vez com conteúdo pronto, após o registro dos itens e equipamentos.</x:v>
       </x:c>
       <x:c r="J1017" s="16" t="str"/>
       <x:c r="K1017" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1018" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1018" ht="34.5" customHeight="1">
       <x:c r="A1018" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="B1018" s="16" t="str">
-        <x:v>Register</x:v>
+        <x:v>Visible</x:v>
       </x:c>
       <x:c r="C1018" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Getter</x:v>
       </x:c>
       <x:c r="D1018" s="16" t="str">
-        <x:v>Register(inst)</x:v>
+        <x:v>get Visible</x:v>
       </x:c>
       <x:c r="E1018" s="16" t="str">
-        <x:v>PrefixLoader</x:v>
+        <x:v>PlayerDrawLayer</x:v>
       </x:c>
       <x:c r="F1018" s="16" t="str">
         <x:v>Não</x:v>
@@ -35668,14 +35668,14 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1018" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>!this.IsHidden</x:v>
       </x:c>
       <x:c r="I1018" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>Consulte a implementação na fonte. Visibilidade própria da camada no desenho atual; um pai oculto também suprime sua execução.</x:v>
       </x:c>
       <x:c r="J1018" s="16" t="str"/>
       <x:c r="K1018" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L34</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PlayerDrawHooks.js#L3</x:v>
       </x:c>
     </x:row>
     <x:row r="1019" ht="21.75" customHeight="1">
@@ -35683,13 +35683,13 @@
         <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1019" s="16" t="str">
-        <x:v>TooltipLines</x:v>
+        <x:v>AllowPrefix</x:v>
       </x:c>
       <x:c r="C1019" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1019" s="16" t="str">
-        <x:v>TooltipLines(item)</x:v>
+        <x:v>AllowPrefix(item, pre)</x:v>
       </x:c>
       <x:c r="E1019" s="16" t="str">
         <x:v>PrefixLoader</x:v>
@@ -35704,11 +35704,11 @@
         <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1019" s="16" t="str">
-        <x:v>As linhas do GetTooltipLines do prefixo do item, ou null.</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1019" s="16" t="str"/>
       <x:c r="K1019" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L132</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L122</x:v>
       </x:c>
     </x:row>
     <x:row r="1020" ht="21.75" customHeight="1">
@@ -35716,13 +35716,13 @@
         <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1020" s="16" t="str">
-        <x:v>VanillaCount</x:v>
+        <x:v>Categories</x:v>
       </x:c>
       <x:c r="C1020" s="16" t="str">
-        <x:v>Getter estático</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1020" s="16" t="str">
-        <x:v>get VanillaCount</x:v>
+        <x:v>Categories(item)</x:v>
       </x:c>
       <x:c r="E1020" s="16" t="str">
         <x:v>PrefixLoader</x:v>
@@ -35737,11 +35737,11 @@
         <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1020" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>As categorias do item; os prefixos do jogo de uma categoria.</x:v>
       </x:c>
       <x:c r="J1020" s="16" t="str"/>
       <x:c r="K1020" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L19</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L83</x:v>
       </x:c>
     </x:row>
     <x:row r="1021" ht="21.75" customHeight="1">
@@ -35749,13 +35749,13 @@
         <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1021" s="16" t="str">
-        <x:v>VanillaPrefixes</x:v>
+        <x:v>GetPrefix</x:v>
       </x:c>
       <x:c r="C1021" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1021" s="16" t="str">
-        <x:v>VanillaPrefixes(category)</x:v>
+        <x:v>GetPrefix(type)</x:v>
       </x:c>
       <x:c r="E1021" s="16" t="str">
         <x:v>PrefixLoader</x:v>
@@ -35767,14 +35767,14 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1021" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>PrefixLoader.ByType.get(type)</x:v>
       </x:c>
       <x:c r="I1021" s="16" t="str">
-        <x:v>As categorias do item; os prefixos do jogo de uma categoria.</x:v>
+        <x:v>O ModPrefix, ou undefined (prefixo do jogo).</x:v>
       </x:c>
       <x:c r="J1021" s="16" t="str"/>
       <x:c r="K1021" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L109</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L26</x:v>
       </x:c>
     </x:row>
     <x:row r="1022" ht="21.75" customHeight="1">
@@ -35782,13 +35782,13 @@
         <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1022" s="16" t="str">
-        <x:v>WantItemHooks</x:v>
+        <x:v>GetPrefixesInCategory</x:v>
       </x:c>
       <x:c r="C1022" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1022" s="16" t="str">
-        <x:v>WantItemHooks(methods)</x:v>
+        <x:v>GetPrefixesInCategory(category)</x:v>
       </x:c>
       <x:c r="E1022" s="16" t="str">
         <x:v>PrefixLoader</x:v>
@@ -35800,28 +35800,28 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1022" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>PrefixLoader.#byCategory.get(category) || []</x:v>
       </x:c>
       <x:c r="I1022" s="16" t="str">
-        <x:v>Os métodos de prefixo que um ModItem/GlobalItem sobrescreve (ChoosePrefix, AllowPrefix...).</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1022" s="16" t="str"/>
       <x:c r="K1022" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1023" ht="34.5" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1023" ht="47.25" customHeight="1">
       <x:c r="A1023" s="16" t="str">
         <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1023" s="16" t="str">
-        <x:v>WantRollable</x:v>
+        <x:v>IsWeaponSubCategory</x:v>
       </x:c>
       <x:c r="C1023" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1023" s="16" t="str">
-        <x:v>WantRollable()</x:v>
+        <x:v>IsWeaponSubCategory(category)</x:v>
       </x:c>
       <x:c r="E1023" s="16" t="str">
         <x:v>PrefixLoader</x:v>
@@ -35833,14 +35833,14 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1023" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>category === PrefixCategory.Melee || category === PrefixCategory.Ranged || category === PrefixCategory.Magic</x:v>
       </x:c>
       <x:c r="I1023" s="16" t="str">
-        <x:v>Item de mod ganha os prefixos das categorias dele (MeleePrefix...): sem isto, as tabelas PrefixLegacy.ItemSets do jogo não o conhecem e ele não ganha nenhum.</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1023" s="16" t="str"/>
       <x:c r="K1023" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L73</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L30</x:v>
       </x:c>
     </x:row>
     <x:row r="1024" ht="21.75" customHeight="1">
@@ -35848,13 +35848,13 @@
         <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1024" s="16" t="str">
-        <x:v>WantRolling</x:v>
+        <x:v>PrefixCount</x:v>
       </x:c>
       <x:c r="C1024" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Getter estático</x:v>
       </x:c>
       <x:c r="D1024" s="16" t="str">
-        <x:v>WantRolling()</x:v>
+        <x:v>get PrefixCount</x:v>
       </x:c>
       <x:c r="E1024" s="16" t="str">
         <x:v>PrefixLoader</x:v>
@@ -35866,31 +35866,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1024" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>PrefixLoader.VanillaCount + PrefixLoader.ByType.size</x:v>
       </x:c>
       <x:c r="I1024" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1024" s="16" t="str"/>
       <x:c r="K1024" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L77</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L24</x:v>
       </x:c>
     </x:row>
     <x:row r="1025" ht="21.75" customHeight="1">
       <x:c r="A1025" s="16" t="str">
-        <x:v>RarityLoader</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1025" s="16" t="str">
-        <x:v>Add</x:v>
+        <x:v>Register</x:v>
       </x:c>
       <x:c r="C1025" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1025" s="16" t="str">
-        <x:v>Add(inst)</x:v>
+        <x:v>Register(inst)</x:v>
       </x:c>
       <x:c r="E1025" s="16" t="str">
-        <x:v>RarityLoader</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="F1025" s="16" t="str">
         <x:v>Não</x:v>
@@ -35906,24 +35906,24 @@
       </x:c>
       <x:c r="J1025" s="16" t="str"/>
       <x:c r="K1025" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/RarityLoader.js#L19</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L34</x:v>
       </x:c>
     </x:row>
     <x:row r="1026" ht="21.75" customHeight="1">
       <x:c r="A1026" s="16" t="str">
-        <x:v>RarityLoader</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1026" s="16" t="str">
-        <x:v>ColorOf</x:v>
+        <x:v>TooltipLines</x:v>
       </x:c>
       <x:c r="C1026" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1026" s="16" t="str">
-        <x:v>ColorOf(type)</x:v>
+        <x:v>TooltipLines(item)</x:v>
       </x:c>
       <x:c r="E1026" s="16" t="str">
-        <x:v>RarityLoader</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="F1026" s="16" t="str">
         <x:v>Não</x:v>
@@ -35935,28 +35935,28 @@
         <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1026" s="16" t="str">
-        <x:v>A cor de uma raridade de mod; branco se o RarityColor falhar.</x:v>
+        <x:v>As linhas do GetTooltipLines do prefixo do item, ou null.</x:v>
       </x:c>
       <x:c r="J1026" s="16" t="str"/>
       <x:c r="K1026" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/RarityLoader.js#L30</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L132</x:v>
       </x:c>
     </x:row>
     <x:row r="1027" ht="21.75" customHeight="1">
       <x:c r="A1027" s="16" t="str">
-        <x:v>RarityLoader</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1027" s="16" t="str">
-        <x:v>GetRarity</x:v>
+        <x:v>VanillaCount</x:v>
       </x:c>
       <x:c r="C1027" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Getter estático</x:v>
       </x:c>
       <x:c r="D1027" s="16" t="str">
-        <x:v>GetRarity(type)</x:v>
+        <x:v>get VanillaCount</x:v>
       </x:c>
       <x:c r="E1027" s="16" t="str">
-        <x:v>RarityLoader</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="F1027" s="16" t="str">
         <x:v>Não</x:v>
@@ -35965,31 +35965,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1027" s="16" t="str">
-        <x:v>RarityLoader.ByType.get(type) || null</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1027" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1027" s="16" t="str"/>
       <x:c r="K1027" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/RarityLoader.js#L27</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L19</x:v>
       </x:c>
     </x:row>
     <x:row r="1028" ht="21.75" customHeight="1">
       <x:c r="A1028" s="16" t="str">
-        <x:v>RarityLoader</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1028" s="16" t="str">
-        <x:v>RarityCount</x:v>
+        <x:v>VanillaPrefixes</x:v>
       </x:c>
       <x:c r="C1028" s="16" t="str">
-        <x:v>Getter estático</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1028" s="16" t="str">
-        <x:v>get RarityCount</x:v>
+        <x:v>VanillaPrefixes(category)</x:v>
       </x:c>
       <x:c r="E1028" s="16" t="str">
-        <x:v>RarityLoader</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="F1028" s="16" t="str">
         <x:v>Não</x:v>
@@ -35998,31 +35998,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1028" s="16" t="str">
-        <x:v>RarityLoader.VanillaCount + RarityLoader.ByType.size</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1028" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>As categorias do item; os prefixos do jogo de uma categoria.</x:v>
       </x:c>
       <x:c r="J1028" s="16" t="str"/>
       <x:c r="K1028" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/RarityLoader.js#L17</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L109</x:v>
       </x:c>
     </x:row>
     <x:row r="1029" ht="21.75" customHeight="1">
       <x:c r="A1029" s="16" t="str">
-        <x:v>SoundEngine</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1029" s="16" t="str">
-        <x:v>FindActiveSound</x:v>
+        <x:v>WantItemHooks</x:v>
       </x:c>
       <x:c r="C1029" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1029" s="16" t="str">
-        <x:v>FindActiveSound(style)</x:v>
+        <x:v>WantItemHooks(methods)</x:v>
       </x:c>
       <x:c r="E1029" s="16" t="str">
-        <x:v>SoundEngine</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="F1029" s="16" t="str">
         <x:v>Não</x:v>
@@ -36034,28 +36034,28 @@
         <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1029" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>Os métodos de prefixo que um ModItem/GlobalItem sobrescreve (ChoosePrefix, AllowPrefix...).</x:v>
       </x:c>
       <x:c r="J1029" s="16" t="str"/>
       <x:c r="K1029" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SoundEngine.js#L19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1030" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L64</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1030" ht="34.5" customHeight="1">
       <x:c r="A1030" s="16" t="str">
-        <x:v>SoundEngine</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1030" s="16" t="str">
-        <x:v>PlaySound</x:v>
+        <x:v>WantRollable</x:v>
       </x:c>
       <x:c r="C1030" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1030" s="16" t="str">
-        <x:v>PlaySound(style, position)</x:v>
+        <x:v>WantRollable()</x:v>
       </x:c>
       <x:c r="E1030" s="16" t="str">
-        <x:v>SoundEngine</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="F1030" s="16" t="str">
         <x:v>Não</x:v>
@@ -36067,28 +36067,28 @@
         <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1030" s="16" t="str">
-        <x:v>Toca agora; som de mod devolve o número (0 = não tocou).</x:v>
+        <x:v>Item de mod ganha os prefixos das categorias dele (MeleePrefix...): sem isto, as tabelas PrefixLegacy.ItemSets do jogo não o conhecem e ele não ganha nenhum.</x:v>
       </x:c>
       <x:c r="J1030" s="16" t="str"/>
       <x:c r="K1030" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SoundEngine.js#L4</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L73</x:v>
       </x:c>
     </x:row>
     <x:row r="1031" ht="21.75" customHeight="1">
       <x:c r="A1031" s="16" t="str">
-        <x:v>SoundEngine</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="B1031" s="16" t="str">
-        <x:v>StopSound</x:v>
+        <x:v>WantRolling</x:v>
       </x:c>
       <x:c r="C1031" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1031" s="16" t="str">
-        <x:v>StopSound(stream)</x:v>
+        <x:v>WantRolling()</x:v>
       </x:c>
       <x:c r="E1031" s="16" t="str">
-        <x:v>SoundEngine</x:v>
+        <x:v>PrefixLoader</x:v>
       </x:c>
       <x:c r="F1031" s="16" t="str">
         <x:v>Não</x:v>
@@ -36104,24 +36104,24 @@
       </x:c>
       <x:c r="J1031" s="16" t="str"/>
       <x:c r="K1031" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SoundEngine.js#L28</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/PrefixLoader.js#L77</x:v>
       </x:c>
     </x:row>
     <x:row r="1032" ht="21.75" customHeight="1">
       <x:c r="A1032" s="16" t="str">
-        <x:v>SoundStyle</x:v>
+        <x:v>RarityLoader</x:v>
       </x:c>
       <x:c r="B1032" s="16" t="str">
-        <x:v>constructor</x:v>
+        <x:v>Add</x:v>
       </x:c>
       <x:c r="C1032" s="16" t="str">
-        <x:v>Construtor</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1032" s="16" t="str">
-        <x:v>constructor(path, options)</x:v>
+        <x:v>Add(inst)</x:v>
       </x:c>
       <x:c r="E1032" s="16" t="str">
-        <x:v>SoundStyle</x:v>
+        <x:v>RarityLoader</x:v>
       </x:c>
       <x:c r="F1032" s="16" t="str">
         <x:v>Não</x:v>
@@ -36130,31 +36130,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1032" s="16" t="str">
-        <x:v>instância</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1032" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1032" s="16" t="str"/>
       <x:c r="K1032" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SoundStyle.js#L5</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/RarityLoader.js#L19</x:v>
       </x:c>
     </x:row>
     <x:row r="1033" ht="21.75" customHeight="1">
       <x:c r="A1033" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>RarityLoader</x:v>
       </x:c>
       <x:c r="B1033" s="16" t="str">
-        <x:v>Active</x:v>
+        <x:v>ColorOf</x:v>
       </x:c>
       <x:c r="C1033" s="16" t="str">
-        <x:v>Getter</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1033" s="16" t="str">
-        <x:v>get Active</x:v>
+        <x:v>ColorOf(type)</x:v>
       </x:c>
       <x:c r="E1033" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>RarityLoader</x:v>
       </x:c>
       <x:c r="F1033" s="16" t="str">
         <x:v>Não</x:v>
@@ -36166,28 +36166,28 @@
         <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1033" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>A cor de uma raridade de mod; branco se o RarityColor falhar.</x:v>
       </x:c>
       <x:c r="J1033" s="16" t="str"/>
       <x:c r="K1033" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L37</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/RarityLoader.js#L30</x:v>
       </x:c>
     </x:row>
     <x:row r="1034" ht="21.75" customHeight="1">
       <x:c r="A1034" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>RarityLoader</x:v>
       </x:c>
       <x:c r="B1034" s="16" t="str">
-        <x:v>Begin</x:v>
+        <x:v>GetRarity</x:v>
       </x:c>
       <x:c r="C1034" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1034" s="16" t="str">
-        <x:v>Begin(info)</x:v>
+        <x:v>GetRarity(type)</x:v>
       </x:c>
       <x:c r="E1034" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>RarityLoader</x:v>
       </x:c>
       <x:c r="F1034" s="16" t="str">
         <x:v>Não</x:v>
@@ -36196,31 +36196,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1034" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>RarityLoader.ByType.get(type) || null</x:v>
       </x:c>
       <x:c r="I1034" s="16" t="str">
-        <x:v>O spawnInfo do sorteio que começa (o SpawnLoader chama antes dos SpawnChance).</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1034" s="16" t="str"/>
       <x:c r="K1034" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L41</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/RarityLoader.js#L27</x:v>
       </x:c>
     </x:row>
     <x:row r="1035" ht="21.75" customHeight="1">
       <x:c r="A1035" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>RarityLoader</x:v>
       </x:c>
       <x:c r="B1035" s="16" t="str">
-        <x:v>BlockWeight</x:v>
+        <x:v>RarityCount</x:v>
       </x:c>
       <x:c r="C1035" s="16" t="str">
-        <x:v>Getter</x:v>
+        <x:v>Getter estático</x:v>
       </x:c>
       <x:c r="D1035" s="16" t="str">
-        <x:v>get BlockWeight</x:v>
+        <x:v>get RarityCount</x:v>
       </x:c>
       <x:c r="E1035" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>RarityLoader</x:v>
       </x:c>
       <x:c r="F1035" s="16" t="str">
         <x:v>Não</x:v>
@@ -36229,31 +36229,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1035" s="16" t="str">
-        <x:v>this.#blockWeight</x:v>
+        <x:v>RarityLoader.VanillaCount + RarityLoader.ByType.size</x:v>
       </x:c>
       <x:c r="I1035" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1035" s="16" t="str"/>
       <x:c r="K1035" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L38</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/Loaders/RarityLoader.js#L17</x:v>
       </x:c>
     </x:row>
     <x:row r="1036" ht="21.75" customHeight="1">
       <x:c r="A1036" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>SoundEngine</x:v>
       </x:c>
       <x:c r="B1036" s="16" t="str">
-        <x:v>Chance</x:v>
+        <x:v>FindActiveSound</x:v>
       </x:c>
       <x:c r="C1036" s="16" t="str">
-        <x:v>Getter</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1036" s="16" t="str">
-        <x:v>get Chance</x:v>
+        <x:v>FindActiveSound(style)</x:v>
       </x:c>
       <x:c r="E1036" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>SoundEngine</x:v>
       </x:c>
       <x:c r="F1036" s="16" t="str">
         <x:v>Não</x:v>
@@ -36269,24 +36269,24 @@
       </x:c>
       <x:c r="J1036" s="16" t="str"/>
       <x:c r="K1036" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L36</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SoundEngine.js#L19</x:v>
       </x:c>
     </x:row>
     <x:row r="1037" ht="21.75" customHeight="1">
       <x:c r="A1037" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>SoundEngine</x:v>
       </x:c>
       <x:c r="B1037" s="16" t="str">
-        <x:v>CheckAll</x:v>
+        <x:v>PlaySound</x:v>
       </x:c>
       <x:c r="C1037" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1037" s="16" t="str">
-        <x:v>CheckAll(info)</x:v>
+        <x:v>PlaySound(style, position)</x:v>
       </x:c>
       <x:c r="E1037" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>SoundEngine</x:v>
       </x:c>
       <x:c r="F1037" s="16" t="str">
         <x:v>Não</x:v>
@@ -36298,28 +36298,28 @@
         <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1037" s="16" t="str">
-        <x:v>Todas as condições no spawnInfo dado, na hora (para testes).</x:v>
+        <x:v>Toca agora; som de mod devolve o número (0 = não tocou).</x:v>
       </x:c>
       <x:c r="J1037" s="16" t="str"/>
       <x:c r="K1037" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L47</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SoundEngine.js#L4</x:v>
       </x:c>
     </x:row>
     <x:row r="1038" ht="21.75" customHeight="1">
       <x:c r="A1038" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>SoundEngine</x:v>
       </x:c>
       <x:c r="B1038" s="16" t="str">
-        <x:v>constructor</x:v>
+        <x:v>StopSound</x:v>
       </x:c>
       <x:c r="C1038" s="16" t="str">
-        <x:v>Construtor</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1038" s="16" t="str">
-        <x:v>constructor(parent, test, blockWeight = 1)</x:v>
+        <x:v>StopSound(stream)</x:v>
       </x:c>
       <x:c r="E1038" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>SoundEngine</x:v>
       </x:c>
       <x:c r="F1038" s="16" t="str">
         <x:v>Não</x:v>
@@ -36328,31 +36328,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1038" s="16" t="str">
-        <x:v>instância</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1038" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1038" s="16" t="str"/>
       <x:c r="K1038" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L24</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SoundEngine.js#L28</x:v>
       </x:c>
     </x:row>
     <x:row r="1039" ht="21.75" customHeight="1">
       <x:c r="A1039" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>SoundStyle</x:v>
       </x:c>
       <x:c r="B1039" s="16" t="str">
-        <x:v>Name</x:v>
+        <x:v>constructor</x:v>
       </x:c>
       <x:c r="C1039" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Construtor</x:v>
       </x:c>
       <x:c r="D1039" s="16" t="str">
-        <x:v>Name(all)</x:v>
+        <x:v>constructor(path, options)</x:v>
       </x:c>
       <x:c r="E1039" s="16" t="str">
-        <x:v>SpawnCondition</x:v>
+        <x:v>SoundStyle</x:v>
       </x:c>
       <x:c r="F1039" s="16" t="str">
         <x:v>Não</x:v>
@@ -36361,31 +36361,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1039" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>instância</x:v>
       </x:c>
       <x:c r="I1039" s="16" t="str">
-        <x:v>Os nomes, para o aviso (depois de criar todas).</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1039" s="16" t="str"/>
       <x:c r="K1039" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L92</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SoundStyle.js#L5</x:v>
       </x:c>
     </x:row>
     <x:row r="1040" ht="21.75" customHeight="1">
       <x:c r="A1040" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="B1040" s="16" t="str">
-        <x:v>Add</x:v>
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="C1040" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Getter</x:v>
       </x:c>
       <x:c r="D1040" s="16" t="str">
-        <x:v>Add(type, weight)</x:v>
+        <x:v>get Active</x:v>
       </x:c>
       <x:c r="E1040" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="F1040" s="16" t="str">
         <x:v>Não</x:v>
@@ -36401,24 +36401,24 @@
       </x:c>
       <x:c r="J1040" s="16" t="str"/>
       <x:c r="K1040" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L9</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L37</x:v>
       </x:c>
     </x:row>
     <x:row r="1041" ht="21.75" customHeight="1">
       <x:c r="A1041" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="B1041" s="16" t="str">
-        <x:v>Choose</x:v>
+        <x:v>Begin</x:v>
       </x:c>
       <x:c r="C1041" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1041" s="16" t="str">
-        <x:v>Choose()</x:v>
+        <x:v>Begin(info)</x:v>
       </x:c>
       <x:c r="E1041" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="F1041" s="16" t="str">
         <x:v>Não</x:v>
@@ -36430,28 +36430,28 @@
         <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1041" s="16" t="str">
-        <x:v>O tipo sorteado pelo Main.rand, ou null com o total 0 (nada nasce). Peso negativo vale 0.</x:v>
+        <x:v>O spawnInfo do sorteio que começa (o SpawnLoader chama antes dos SpawnChance).</x:v>
       </x:c>
       <x:c r="J1041" s="16" t="str"/>
       <x:c r="K1041" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L28</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L41</x:v>
       </x:c>
     </x:row>
     <x:row r="1042" ht="21.75" customHeight="1">
       <x:c r="A1042" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="B1042" s="16" t="str">
-        <x:v>Clear</x:v>
+        <x:v>BlockWeight</x:v>
       </x:c>
       <x:c r="C1042" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Getter</x:v>
       </x:c>
       <x:c r="D1042" s="16" t="str">
-        <x:v>Clear()</x:v>
+        <x:v>get BlockWeight</x:v>
       </x:c>
       <x:c r="E1042" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="F1042" s="16" t="str">
         <x:v>Não</x:v>
@@ -36460,31 +36460,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1042" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>this.#blockWeight</x:v>
       </x:c>
       <x:c r="I1042" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1042" s="16" t="str"/>
       <x:c r="K1042" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L22</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L38</x:v>
       </x:c>
     </x:row>
     <x:row r="1043" ht="21.75" customHeight="1">
       <x:c r="A1043" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="B1043" s="16" t="str">
-        <x:v>ContainsKey</x:v>
+        <x:v>Chance</x:v>
       </x:c>
       <x:c r="C1043" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Getter</x:v>
       </x:c>
       <x:c r="D1043" s="16" t="str">
-        <x:v>ContainsKey(type)</x:v>
+        <x:v>get Chance</x:v>
       </x:c>
       <x:c r="E1043" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="F1043" s="16" t="str">
         <x:v>Não</x:v>
@@ -36493,31 +36493,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1043" s="16" t="str">
-        <x:v>Object.prototype.hasOwnProperty.call(this, type)</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1043" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1043" s="16" t="str"/>
       <x:c r="K1043" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L14</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L36</x:v>
       </x:c>
     </x:row>
     <x:row r="1044" ht="21.75" customHeight="1">
       <x:c r="A1044" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="B1044" s="16" t="str">
-        <x:v>Count</x:v>
+        <x:v>CheckAll</x:v>
       </x:c>
       <x:c r="C1044" s="16" t="str">
-        <x:v>Getter</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1044" s="16" t="str">
-        <x:v>get Count</x:v>
+        <x:v>CheckAll(info)</x:v>
       </x:c>
       <x:c r="E1044" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="F1044" s="16" t="str">
         <x:v>Não</x:v>
@@ -36526,31 +36526,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1044" s="16" t="str">
-        <x:v>Object.keys(this).length</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1044" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>Todas as condições no spawnInfo dado, na hora (para testes).</x:v>
       </x:c>
       <x:c r="J1044" s="16" t="str"/>
       <x:c r="K1044" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L6</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L47</x:v>
       </x:c>
     </x:row>
     <x:row r="1045" ht="21.75" customHeight="1">
       <x:c r="A1045" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="B1045" s="16" t="str">
-        <x:v>Keys</x:v>
+        <x:v>constructor</x:v>
       </x:c>
       <x:c r="C1045" s="16" t="str">
-        <x:v>Getter</x:v>
+        <x:v>Construtor</x:v>
       </x:c>
       <x:c r="D1045" s="16" t="str">
-        <x:v>get Keys</x:v>
+        <x:v>constructor(parent, test, blockWeight = 1)</x:v>
       </x:c>
       <x:c r="E1045" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="F1045" s="16" t="str">
         <x:v>Não</x:v>
@@ -36559,31 +36559,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1045" s="16" t="str">
-        <x:v>Object.keys(this).map(Number)</x:v>
+        <x:v>instância</x:v>
       </x:c>
       <x:c r="I1045" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1045" s="16" t="str"/>
       <x:c r="K1045" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L7</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L24</x:v>
       </x:c>
     </x:row>
     <x:row r="1046" ht="21.75" customHeight="1">
       <x:c r="A1046" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="B1046" s="16" t="str">
-        <x:v>Remove</x:v>
+        <x:v>Name</x:v>
       </x:c>
       <x:c r="C1046" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1046" s="16" t="str">
-        <x:v>Remove(type)</x:v>
+        <x:v>Name(all)</x:v>
       </x:c>
       <x:c r="E1046" s="16" t="str">
-        <x:v>SpawnPool</x:v>
+        <x:v>SpawnCondition</x:v>
       </x:c>
       <x:c r="F1046" s="16" t="str">
         <x:v>Não</x:v>
@@ -36595,28 +36595,28 @@
         <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1046" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>Os nomes, para o aviso (depois de criar todas).</x:v>
       </x:c>
       <x:c r="J1046" s="16" t="str"/>
       <x:c r="K1046" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1047" ht="34.5" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnCondition.js#L92</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1047" ht="21.75" customHeight="1">
       <x:c r="A1047" s="16" t="str">
-        <x:v>StatInheritanceData</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="B1047" s="16" t="str">
-        <x:v>constructor</x:v>
+        <x:v>Add</x:v>
       </x:c>
       <x:c r="C1047" s="16" t="str">
-        <x:v>Construtor</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1047" s="16" t="str">
-        <x:v>constructor(damageInheritance = 0, critChanceInheritance = 0, attackSpeedInheritance = 0, armorPenInheritance = 0, knockbackInheritance = 0)</x:v>
+        <x:v>Add(type, weight)</x:v>
       </x:c>
       <x:c r="E1047" s="16" t="str">
-        <x:v>StatInheritanceData</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="F1047" s="16" t="str">
         <x:v>Não</x:v>
@@ -36625,31 +36625,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1047" s="16" t="str">
-        <x:v>instância</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1047" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1047" s="16" t="str"/>
       <x:c r="K1047" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatInheritanceData.js#L5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1048" ht="34.5" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1048" ht="21.75" customHeight="1">
       <x:c r="A1048" s="16" t="str">
-        <x:v>StatInheritanceData</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="B1048" s="16" t="str">
-        <x:v>Full</x:v>
+        <x:v>Choose</x:v>
       </x:c>
       <x:c r="C1048" s="16" t="str">
-        <x:v>Getter estático</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1048" s="16" t="str">
-        <x:v>get Full</x:v>
+        <x:v>Choose()</x:v>
       </x:c>
       <x:c r="E1048" s="16" t="str">
-        <x:v>StatInheritanceData</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="F1048" s="16" t="str">
         <x:v>Não</x:v>
@@ -36658,31 +36658,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1048" s="16" t="str">
-        <x:v>new StatInheritanceData(1, 1, 1, 1, 1)</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1048" s="16" t="str">
-        <x:v>Um novo a cada leitura: o Full with { attackSpeedInheritance = 0 } do C# vira Object.assign(StatInheritanceData.Full, { attackSpeedInheritance: 0 }).</x:v>
+        <x:v>O tipo sorteado pelo Main.rand, ou null com o total 0 (nada nasce). Peso negativo vale 0.</x:v>
       </x:c>
       <x:c r="J1048" s="16" t="str"/>
       <x:c r="K1048" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatInheritanceData.js#L24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1049" ht="47.25" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1049" ht="21.75" customHeight="1">
       <x:c r="A1049" s="16" t="str">
-        <x:v>StatInheritanceData</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="B1049" s="16" t="str">
-        <x:v>IsNone</x:v>
+        <x:v>Clear</x:v>
       </x:c>
       <x:c r="C1049" s="16" t="str">
-        <x:v>Getter</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1049" s="16" t="str">
-        <x:v>get IsNone</x:v>
+        <x:v>Clear()</x:v>
       </x:c>
       <x:c r="E1049" s="16" t="str">
-        <x:v>StatInheritanceData</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="F1049" s="16" t="str">
         <x:v>Não</x:v>
@@ -36691,31 +36691,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1049" s="16" t="str">
-        <x:v>!this.damageInheritance &amp;&amp; !this.critChanceInheritance &amp;&amp; !this.attackSpeedInheritance &amp;&amp; !this.armorPenInheritance &amp;&amp; !this.knockbackInheritance</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1049" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1049" s="16" t="str"/>
       <x:c r="K1049" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatInheritanceData.js#L27</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L22</x:v>
       </x:c>
     </x:row>
     <x:row r="1050" ht="21.75" customHeight="1">
       <x:c r="A1050" s="16" t="str">
-        <x:v>StatInheritanceData</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="B1050" s="16" t="str">
-        <x:v>None</x:v>
+        <x:v>ContainsKey</x:v>
       </x:c>
       <x:c r="C1050" s="16" t="str">
-        <x:v>Getter estático</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1050" s="16" t="str">
-        <x:v>get None</x:v>
+        <x:v>ContainsKey(type)</x:v>
       </x:c>
       <x:c r="E1050" s="16" t="str">
-        <x:v>StatInheritanceData</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="F1050" s="16" t="str">
         <x:v>Não</x:v>
@@ -36724,31 +36724,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1050" s="16" t="str">
-        <x:v>new StatInheritanceData()</x:v>
+        <x:v>Object.prototype.hasOwnProperty.call(this, type)</x:v>
       </x:c>
       <x:c r="I1050" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1050" s="16" t="str"/>
       <x:c r="K1050" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatInheritanceData.js#L25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1051" ht="34.5" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1051" ht="21.75" customHeight="1">
       <x:c r="A1051" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="B1051" s="16" t="str">
-        <x:v>ApplyTo</x:v>
+        <x:v>Count</x:v>
       </x:c>
       <x:c r="C1051" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Getter</x:v>
       </x:c>
       <x:c r="D1051" s="16" t="str">
-        <x:v>ApplyTo(baseValue)</x:v>
+        <x:v>get Count</x:v>
       </x:c>
       <x:c r="E1051" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="F1051" s="16" t="str">
         <x:v>Não</x:v>
@@ -36757,31 +36757,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1051" s="16" t="str">
-        <x:v>(baseValue + this.Base) * this.Additive * this.Multiplicative + this.Flat</x:v>
+        <x:v>Object.keys(this).length</x:v>
       </x:c>
       <x:c r="I1051" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1051" s="16" t="str"/>
       <x:c r="K1051" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1052" ht="34.5" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1052" ht="21.75" customHeight="1">
       <x:c r="A1052" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="B1052" s="16" t="str">
-        <x:v>Clone</x:v>
+        <x:v>Keys</x:v>
       </x:c>
       <x:c r="C1052" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Getter</x:v>
       </x:c>
       <x:c r="D1052" s="16" t="str">
-        <x:v>Clone()</x:v>
+        <x:v>get Keys</x:v>
       </x:c>
       <x:c r="E1052" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="F1052" s="16" t="str">
         <x:v>Não</x:v>
@@ -36790,31 +36790,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1052" s="16" t="str">
-        <x:v>new StatModifier(this.Additive, this.Multiplicative, this.Flat, this.Base)</x:v>
+        <x:v>Object.keys(this).map(Number)</x:v>
       </x:c>
       <x:c r="I1052" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1052" s="16" t="str"/>
       <x:c r="K1052" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L33</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1053" ht="47.25" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1053" ht="21.75" customHeight="1">
       <x:c r="A1053" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="B1053" s="16" t="str">
-        <x:v>CombineWith</x:v>
+        <x:v>Remove</x:v>
       </x:c>
       <x:c r="C1053" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1053" s="16" t="str">
-        <x:v>CombineWith(m)</x:v>
+        <x:v>Remove(type)</x:v>
       </x:c>
       <x:c r="E1053" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>SpawnPool</x:v>
       </x:c>
       <x:c r="F1053" s="16" t="str">
         <x:v>Não</x:v>
@@ -36823,19 +36823,19 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1053" s="16" t="str">
-        <x:v>new StatModifier(this.Additive + m.Additive - 1, this.Multiplicative * m.Multiplicative, this.Flat + m.Flat, this.Base + m.Base)</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1053" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1053" s="16" t="str"/>
       <x:c r="K1053" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1054" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/SpawnPool.js#L16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1054" ht="34.5" customHeight="1">
       <x:c r="A1054" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>StatInheritanceData</x:v>
       </x:c>
       <x:c r="B1054" s="16" t="str">
         <x:v>constructor</x:v>
@@ -36844,10 +36844,10 @@
         <x:v>Construtor</x:v>
       </x:c>
       <x:c r="D1054" s="16" t="str">
-        <x:v>constructor(additive = 1, multiplicative = 1, flat = 0, base = 0)</x:v>
+        <x:v>constructor(damageInheritance = 0, critChanceInheritance = 0, attackSpeedInheritance = 0, armorPenInheritance = 0, knockbackInheritance = 0)</x:v>
       </x:c>
       <x:c r="E1054" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>StatInheritanceData</x:v>
       </x:c>
       <x:c r="F1054" s="16" t="str">
         <x:v>Não</x:v>
@@ -36863,24 +36863,24 @@
       </x:c>
       <x:c r="J1054" s="16" t="str"/>
       <x:c r="K1054" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1055" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatInheritanceData.js#L5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1055" ht="34.5" customHeight="1">
       <x:c r="A1055" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>StatInheritanceData</x:v>
       </x:c>
       <x:c r="B1055" s="16" t="str">
-        <x:v>Default</x:v>
+        <x:v>Full</x:v>
       </x:c>
       <x:c r="C1055" s="16" t="str">
         <x:v>Getter estático</x:v>
       </x:c>
       <x:c r="D1055" s="16" t="str">
-        <x:v>get Default</x:v>
+        <x:v>get Full</x:v>
       </x:c>
       <x:c r="E1055" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>StatInheritanceData</x:v>
       </x:c>
       <x:c r="F1055" s="16" t="str">
         <x:v>Não</x:v>
@@ -36889,31 +36889,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1055" s="16" t="str">
-        <x:v>new StatModifier()</x:v>
+        <x:v>new StatInheritanceData(1, 1, 1, 1, 1)</x:v>
       </x:c>
       <x:c r="I1055" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>Um novo a cada leitura: o Full with { attackSpeedInheritance = 0 } do C# vira Object.assign(StatInheritanceData.Full, { attackSpeedInheritance: 0 }).</x:v>
       </x:c>
       <x:c r="J1055" s="16" t="str"/>
       <x:c r="K1055" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L13</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatInheritanceData.js#L24</x:v>
       </x:c>
     </x:row>
     <x:row r="1056" ht="47.25" customHeight="1">
       <x:c r="A1056" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>StatInheritanceData</x:v>
       </x:c>
       <x:c r="B1056" s="16" t="str">
-        <x:v>Equals</x:v>
+        <x:v>IsNone</x:v>
       </x:c>
       <x:c r="C1056" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Getter</x:v>
       </x:c>
       <x:c r="D1056" s="16" t="str">
-        <x:v>Equals(m)</x:v>
+        <x:v>get IsNone</x:v>
       </x:c>
       <x:c r="E1056" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>StatInheritanceData</x:v>
       </x:c>
       <x:c r="F1056" s="16" t="str">
         <x:v>Não</x:v>
@@ -36922,31 +36922,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1056" s="16" t="str">
-        <x:v>!!m &amp;&amp; this.Additive === m.Additive &amp;&amp; this.Multiplicative === m.Multiplicative &amp;&amp; this.Flat === m.Flat &amp;&amp; this.Base === m.Base</x:v>
+        <x:v>!this.damageInheritance &amp;&amp; !this.critChanceInheritance &amp;&amp; !this.attackSpeedInheritance &amp;&amp; !this.armorPenInheritance &amp;&amp; !this.knockbackInheritance</x:v>
       </x:c>
       <x:c r="I1056" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1056" s="16" t="str"/>
       <x:c r="K1056" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L37</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1057" ht="34.5" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatInheritanceData.js#L27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1057" ht="21.75" customHeight="1">
       <x:c r="A1057" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>StatInheritanceData</x:v>
       </x:c>
       <x:c r="B1057" s="16" t="str">
-        <x:v>ForValue</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="C1057" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Getter estático</x:v>
       </x:c>
       <x:c r="D1057" s="16" t="str">
-        <x:v>ForValue(value)</x:v>
+        <x:v>get None</x:v>
       </x:c>
       <x:c r="E1057" s="16" t="str">
-        <x:v>StatModifier</x:v>
+        <x:v>StatInheritanceData</x:v>
       </x:c>
       <x:c r="F1057" s="16" t="str">
         <x:v>Não</x:v>
@@ -36955,28 +36955,28 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1057" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>new StatInheritanceData()</x:v>
       </x:c>
       <x:c r="I1057" s="16" t="str">
-        <x:v>O damage dos ModifyWeaponDamage: vale como número (return damage  2, o jeito de antes) e como StatModifier (damage.Additive += 0.1, o do tModLoader). O que o mod devolver em número ganha; senão vale o modificador.</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1057" s="16" t="str"/>
       <x:c r="K1057" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L45</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1058" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatInheritanceData.js#L25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1058" ht="34.5" customHeight="1">
       <x:c r="A1058" s="16" t="str">
         <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="B1058" s="16" t="str">
-        <x:v>Resolve</x:v>
+        <x:v>ApplyTo</x:v>
       </x:c>
       <x:c r="C1058" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1058" s="16" t="str">
-        <x:v>Resolve(result, modifier, value)</x:v>
+        <x:v>ApplyTo(baseValue)</x:v>
       </x:c>
       <x:c r="E1058" s="16" t="str">
         <x:v>StatModifier</x:v>
@@ -36988,28 +36988,28 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1058" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>(baseValue + this.Base) * this.Additive * this.Multiplicative + this.Flat</x:v>
       </x:c>
       <x:c r="I1058" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1058" s="16" t="str"/>
       <x:c r="K1058" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L51</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1059" ht="47.25" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1059" ht="34.5" customHeight="1">
       <x:c r="A1059" s="16" t="str">
         <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="B1059" s="16" t="str">
-        <x:v>Scale</x:v>
+        <x:v>Clone</x:v>
       </x:c>
       <x:c r="C1059" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1059" s="16" t="str">
-        <x:v>Scale(scale)</x:v>
+        <x:v>Clone()</x:v>
       </x:c>
       <x:c r="E1059" s="16" t="str">
         <x:v>StatModifier</x:v>
@@ -37021,28 +37021,28 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1059" s="16" t="str">
-        <x:v>new StatModifier(1 + (this.Additive - 1) * scale, 1 + (this.Multiplicative - 1) * scale, this.Flat * scale, this.Base * scale)</x:v>
+        <x:v>new StatModifier(this.Additive, this.Multiplicative, this.Flat, this.Base)</x:v>
       </x:c>
       <x:c r="I1059" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1059" s="16" t="str"/>
       <x:c r="K1059" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1060" ht="34.5" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L33</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1060" ht="47.25" customHeight="1">
       <x:c r="A1060" s="16" t="str">
         <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="B1060" s="16" t="str">
-        <x:v>Undo</x:v>
+        <x:v>CombineWith</x:v>
       </x:c>
       <x:c r="C1060" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1060" s="16" t="str">
-        <x:v>Undo(currentValue)</x:v>
+        <x:v>CombineWith(m)</x:v>
       </x:c>
       <x:c r="E1060" s="16" t="str">
         <x:v>StatModifier</x:v>
@@ -37054,31 +37054,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1060" s="16" t="str">
-        <x:v>(currentValue - this.Flat) / (this.Multiplicative * this.Additive) - this.Base</x:v>
+        <x:v>new StatModifier(this.Additive + m.Additive - 1, this.Multiplicative * m.Multiplicative, this.Flat + m.Flat, this.Base + m.Base)</x:v>
       </x:c>
       <x:c r="I1060" s="16" t="str">
         <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1060" s="16" t="str"/>
       <x:c r="K1060" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L29</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L19</x:v>
       </x:c>
     </x:row>
     <x:row r="1061" ht="21.75" customHeight="1">
       <x:c r="A1061" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="B1061" s="16" t="str">
-        <x:v>Add</x:v>
+        <x:v>constructor</x:v>
       </x:c>
       <x:c r="C1061" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Construtor</x:v>
       </x:c>
       <x:c r="D1061" s="16" t="str">
-        <x:v>Add(key, value)</x:v>
+        <x:v>constructor(additive = 1, multiplicative = 1, flat = 0, base = 0)</x:v>
       </x:c>
       <x:c r="E1061" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="F1061" s="16" t="str">
         <x:v>Não</x:v>
@@ -37087,31 +37087,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1061" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>instância</x:v>
       </x:c>
       <x:c r="I1061" s="16" t="str">
-        <x:v>Escrever e apagar.</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1061" s="16" t="str"/>
       <x:c r="K1061" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L7</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L6</x:v>
       </x:c>
     </x:row>
     <x:row r="1062" ht="21.75" customHeight="1">
       <x:c r="A1062" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="B1062" s="16" t="str">
-        <x:v>ContainsKey</x:v>
+        <x:v>Default</x:v>
       </x:c>
       <x:c r="C1062" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Getter estático</x:v>
       </x:c>
       <x:c r="D1062" s="16" t="str">
-        <x:v>ContainsKey(key)</x:v>
+        <x:v>get Default</x:v>
       </x:c>
       <x:c r="E1062" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="F1062" s="16" t="str">
         <x:v>Não</x:v>
@@ -37120,31 +37120,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1062" s="16" t="str">
-        <x:v>Object.prototype.hasOwnProperty.call(this, key)</x:v>
+        <x:v>new StatModifier()</x:v>
       </x:c>
       <x:c r="I1062" s="16" t="str">
-        <x:v>A chave foi salva?</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1062" s="16" t="str"/>
       <x:c r="K1062" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1063" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1063" ht="47.25" customHeight="1">
       <x:c r="A1063" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="B1063" s="16" t="str">
-        <x:v>Count</x:v>
+        <x:v>Equals</x:v>
       </x:c>
       <x:c r="C1063" s="16" t="str">
-        <x:v>Getter</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1063" s="16" t="str">
-        <x:v>get Count</x:v>
+        <x:v>Equals(m)</x:v>
       </x:c>
       <x:c r="E1063" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="F1063" s="16" t="str">
         <x:v>Não</x:v>
@@ -37153,31 +37153,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1063" s="16" t="str">
-        <x:v>Object.keys(this).length</x:v>
+        <x:v>!!m &amp;&amp; this.Additive === m.Additive &amp;&amp; this.Multiplicative === m.Multiplicative &amp;&amp; this.Flat === m.Flat &amp;&amp; this.Base === m.Base</x:v>
       </x:c>
       <x:c r="I1063" s="16" t="str">
-        <x:v>Quantas chaves.</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1063" s="16" t="str"/>
       <x:c r="K1063" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L2</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L37</x:v>
       </x:c>
     </x:row>
     <x:row r="1064" ht="34.5" customHeight="1">
       <x:c r="A1064" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="B1064" s="16" t="str">
-        <x:v>from</x:v>
+        <x:v>ForValue</x:v>
       </x:c>
       <x:c r="C1064" s="16" t="str">
         <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1064" s="16" t="str">
-        <x:v>from(data)</x:v>
+        <x:v>ForValue(value)</x:v>
       </x:c>
       <x:c r="E1064" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="F1064" s="16" t="str">
         <x:v>Não</x:v>
@@ -37186,31 +37186,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1064" s="16" t="str">
-        <x:v>Object.assign(new TagCompound(), data &amp;&amp; typeof data === 'object' ? data : {})</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1064" s="16" t="str">
-        <x:v>Um TagCompound com os campos do objeto.</x:v>
+        <x:v>O damage dos ModifyWeaponDamage: vale como número (return damage  2, o jeito de antes) e como StatModifier (damage.Additive += 0.1, o do tModLoader). O que o mod devolver em número ganha; senão vale o modificador.</x:v>
       </x:c>
       <x:c r="J1064" s="16" t="str"/>
       <x:c r="K1064" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L17</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L45</x:v>
       </x:c>
     </x:row>
     <x:row r="1065" ht="21.75" customHeight="1">
       <x:c r="A1065" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="B1065" s="16" t="str">
-        <x:v>Get</x:v>
+        <x:v>Resolve</x:v>
       </x:c>
       <x:c r="C1065" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1065" s="16" t="str">
-        <x:v>Get(key, fallback)</x:v>
+        <x:v>Resolve(result, modifier, value)</x:v>
       </x:c>
       <x:c r="E1065" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="F1065" s="16" t="str">
         <x:v>Não</x:v>
@@ -37219,31 +37219,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1065" s="16" t="str">
-        <x:v>this.ContainsKey(key) ? this[key] : fallback</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1065" s="16" t="str">
-        <x:v>O valor, ou o padrão.</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1065" s="16" t="str"/>
       <x:c r="K1065" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1066" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L51</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1066" ht="47.25" customHeight="1">
       <x:c r="A1066" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="B1066" s="16" t="str">
-        <x:v>GetBool</x:v>
+        <x:v>Scale</x:v>
       </x:c>
       <x:c r="C1066" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1066" s="16" t="str">
-        <x:v>GetBool(key)</x:v>
+        <x:v>Scale(scale)</x:v>
       </x:c>
       <x:c r="E1066" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="F1066" s="16" t="str">
         <x:v>Não</x:v>
@@ -37252,31 +37252,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1066" s="16" t="str">
-        <x:v>!!this.Get(key, false)</x:v>
+        <x:v>new StatModifier(1 + (this.Additive - 1) * scale, 1 + (this.Multiplicative - 1) * scale, this.Flat * scale, this.Base * scale)</x:v>
       </x:c>
       <x:c r="I1066" s="16" t="str">
-        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1066" s="16" t="str"/>
       <x:c r="K1066" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1067" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1067" ht="34.5" customHeight="1">
       <x:c r="A1067" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="B1067" s="16" t="str">
-        <x:v>GetCompound</x:v>
+        <x:v>Undo</x:v>
       </x:c>
       <x:c r="C1067" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1067" s="16" t="str">
-        <x:v>GetCompound(key)</x:v>
+        <x:v>Undo(currentValue)</x:v>
       </x:c>
       <x:c r="E1067" s="16" t="str">
-        <x:v>TagCompound</x:v>
+        <x:v>StatModifier</x:v>
       </x:c>
       <x:c r="F1067" s="16" t="str">
         <x:v>Não</x:v>
@@ -37285,14 +37285,14 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1067" s="16" t="str">
-        <x:v>TagCompound.from(this[key])</x:v>
+        <x:v>(currentValue - this.Flat) / (this.Multiplicative * this.Additive) - this.Base</x:v>
       </x:c>
       <x:c r="I1067" s="16" t="str">
-        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
+        <x:v>Consulte a implementação na fonte.</x:v>
       </x:c>
       <x:c r="J1067" s="16" t="str"/>
       <x:c r="K1067" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L15</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/StatModifier.js#L29</x:v>
       </x:c>
     </x:row>
     <x:row r="1068" ht="21.75" customHeight="1">
@@ -37300,13 +37300,13 @@
         <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="B1068" s="16" t="str">
-        <x:v>GetFloat</x:v>
+        <x:v>Add</x:v>
       </x:c>
       <x:c r="C1068" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1068" s="16" t="str">
-        <x:v>GetFloat(key)</x:v>
+        <x:v>Add(key, value)</x:v>
       </x:c>
       <x:c r="E1068" s="16" t="str">
         <x:v>TagCompound</x:v>
@@ -37318,14 +37318,14 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1068" s="16" t="str">
-        <x:v>Number(this.Get(key, 0))</x:v>
+        <x:v>Consultar fonte</x:v>
       </x:c>
       <x:c r="I1068" s="16" t="str">
-        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
+        <x:v>Escrever e apagar.</x:v>
       </x:c>
       <x:c r="J1068" s="16" t="str"/>
       <x:c r="K1068" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L12</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L7</x:v>
       </x:c>
     </x:row>
     <x:row r="1069" ht="21.75" customHeight="1">
@@ -37333,13 +37333,13 @@
         <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="B1069" s="16" t="str">
-        <x:v>GetInt</x:v>
+        <x:v>ContainsKey</x:v>
       </x:c>
       <x:c r="C1069" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1069" s="16" t="str">
-        <x:v>GetInt(key)</x:v>
+        <x:v>ContainsKey(key)</x:v>
       </x:c>
       <x:c r="E1069" s="16" t="str">
         <x:v>TagCompound</x:v>
@@ -37351,14 +37351,14 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1069" s="16" t="str">
-        <x:v>Number(this.Get(key, 0)) | 0</x:v>
+        <x:v>Object.prototype.hasOwnProperty.call(this, key)</x:v>
       </x:c>
       <x:c r="I1069" s="16" t="str">
-        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
+        <x:v>A chave foi salva?</x:v>
       </x:c>
       <x:c r="J1069" s="16" t="str"/>
       <x:c r="K1069" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L11</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L4</x:v>
       </x:c>
     </x:row>
     <x:row r="1070" ht="21.75" customHeight="1">
@@ -37366,13 +37366,13 @@
         <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="B1070" s="16" t="str">
-        <x:v>GetList</x:v>
+        <x:v>Count</x:v>
       </x:c>
       <x:c r="C1070" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Getter</x:v>
       </x:c>
       <x:c r="D1070" s="16" t="str">
-        <x:v>GetList(key)</x:v>
+        <x:v>get Count</x:v>
       </x:c>
       <x:c r="E1070" s="16" t="str">
         <x:v>TagCompound</x:v>
@@ -37384,28 +37384,28 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1070" s="16" t="str">
-        <x:v>Array.isArray(this[key]) ? this[key] : []</x:v>
+        <x:v>Object.keys(this).length</x:v>
       </x:c>
       <x:c r="I1070" s="16" t="str">
-        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
+        <x:v>Quantas chaves.</x:v>
       </x:c>
       <x:c r="J1070" s="16" t="str"/>
       <x:c r="K1070" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="1071" ht="21.75" customHeight="1">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1071" ht="34.5" customHeight="1">
       <x:c r="A1071" s="16" t="str">
         <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="B1071" s="16" t="str">
-        <x:v>GetString</x:v>
+        <x:v>from</x:v>
       </x:c>
       <x:c r="C1071" s="16" t="str">
-        <x:v>Instância</x:v>
+        <x:v>Estático</x:v>
       </x:c>
       <x:c r="D1071" s="16" t="str">
-        <x:v>GetString(key)</x:v>
+        <x:v>from(data)</x:v>
       </x:c>
       <x:c r="E1071" s="16" t="str">
         <x:v>TagCompound</x:v>
@@ -37417,14 +37417,14 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1071" s="16" t="str">
-        <x:v>String(this.Get(key, ''))</x:v>
+        <x:v>Object.assign(new TagCompound(), data &amp;&amp; typeof data === 'object' ? data : {})</x:v>
       </x:c>
       <x:c r="I1071" s="16" t="str">
-        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
+        <x:v>Um TagCompound com os campos do objeto.</x:v>
       </x:c>
       <x:c r="J1071" s="16" t="str"/>
       <x:c r="K1071" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L13</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L17</x:v>
       </x:c>
     </x:row>
     <x:row r="1072" ht="21.75" customHeight="1">
@@ -37432,13 +37432,13 @@
         <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="B1072" s="16" t="str">
-        <x:v>Remove</x:v>
+        <x:v>Get</x:v>
       </x:c>
       <x:c r="C1072" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1072" s="16" t="str">
-        <x:v>Remove(key)</x:v>
+        <x:v>Get(key, fallback)</x:v>
       </x:c>
       <x:c r="E1072" s="16" t="str">
         <x:v>TagCompound</x:v>
@@ -37450,14 +37450,14 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1072" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>this.ContainsKey(key) ? this[key] : fallback</x:v>
       </x:c>
       <x:c r="I1072" s="16" t="str">
-        <x:v>Escrever e apagar.</x:v>
+        <x:v>O valor, ou o padrão.</x:v>
       </x:c>
       <x:c r="J1072" s="16" t="str"/>
       <x:c r="K1072" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L8</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L5</x:v>
       </x:c>
     </x:row>
     <x:row r="1073" ht="21.75" customHeight="1">
@@ -37465,13 +37465,13 @@
         <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="B1073" s="16" t="str">
-        <x:v>Set</x:v>
+        <x:v>GetBool</x:v>
       </x:c>
       <x:c r="C1073" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1073" s="16" t="str">
-        <x:v>Set(key, value)</x:v>
+        <x:v>GetBool(key)</x:v>
       </x:c>
       <x:c r="E1073" s="16" t="str">
         <x:v>TagCompound</x:v>
@@ -37483,31 +37483,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1073" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>!!this.Get(key, false)</x:v>
       </x:c>
       <x:c r="I1073" s="16" t="str">
-        <x:v>Escrever e apagar.</x:v>
+        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
       </x:c>
       <x:c r="J1073" s="16" t="str"/>
       <x:c r="K1073" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L6</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L10</x:v>
       </x:c>
     </x:row>
     <x:row r="1074" ht="21.75" customHeight="1">
       <x:c r="A1074" s="16" t="str">
-        <x:v>TooltipLine</x:v>
+        <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="B1074" s="16" t="str">
-        <x:v>colorTag</x:v>
+        <x:v>GetCompound</x:v>
       </x:c>
       <x:c r="C1074" s="16" t="str">
-        <x:v>Estático</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1074" s="16" t="str">
-        <x:v>colorTag(text, color)</x:v>
+        <x:v>GetCompound(key)</x:v>
       </x:c>
       <x:c r="E1074" s="16" t="str">
-        <x:v>TooltipLine</x:v>
+        <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="F1074" s="16" t="str">
         <x:v>Não</x:v>
@@ -37516,31 +37516,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1074" s="16" t="str">
-        <x:v>'[c/' + TooltipLoader.Hex(color) + ':' + text + ']'</x:v>
+        <x:v>TagCompound.from(this[key])</x:v>
       </x:c>
       <x:c r="I1074" s="16" t="str">
-        <x:v>'[c/RRGGBB:texto]' para pintar um trecho.</x:v>
+        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
       </x:c>
       <x:c r="J1074" s="16" t="str"/>
       <x:c r="K1074" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TooltipLine.js#L20</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L15</x:v>
       </x:c>
     </x:row>
     <x:row r="1075" ht="21.75" customHeight="1">
       <x:c r="A1075" s="16" t="str">
-        <x:v>TooltipLine</x:v>
+        <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="B1075" s="16" t="str">
-        <x:v>constructor</x:v>
+        <x:v>GetFloat</x:v>
       </x:c>
       <x:c r="C1075" s="16" t="str">
-        <x:v>Construtor</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1075" s="16" t="str">
-        <x:v>constructor(...args)</x:v>
+        <x:v>GetFloat(key)</x:v>
       </x:c>
       <x:c r="E1075" s="16" t="str">
-        <x:v>TooltipLine</x:v>
+        <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="F1075" s="16" t="str">
         <x:v>Não</x:v>
@@ -37549,31 +37549,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1075" s="16" t="str">
-        <x:v>instância</x:v>
+        <x:v>Number(this.Get(key, 0))</x:v>
       </x:c>
       <x:c r="I1075" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
       </x:c>
       <x:c r="J1075" s="16" t="str"/>
       <x:c r="K1075" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TooltipLine.js#L5</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L12</x:v>
       </x:c>
     </x:row>
     <x:row r="1076" ht="21.75" customHeight="1">
       <x:c r="A1076" s="16" t="str">
-        <x:v>TooltipLine</x:v>
+        <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="B1076" s="16" t="str">
-        <x:v>Hide</x:v>
+        <x:v>GetInt</x:v>
       </x:c>
       <x:c r="C1076" s="16" t="str">
         <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1076" s="16" t="str">
-        <x:v>Hide()</x:v>
+        <x:v>GetInt(key)</x:v>
       </x:c>
       <x:c r="E1076" s="16" t="str">
-        <x:v>TooltipLine</x:v>
+        <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="F1076" s="16" t="str">
         <x:v>Não</x:v>
@@ -37582,31 +37582,31 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1076" s="16" t="str">
-        <x:v>Consultar fonte</x:v>
+        <x:v>Number(this.Get(key, 0)) | 0</x:v>
       </x:c>
       <x:c r="I1076" s="16" t="str">
-        <x:v>Hide() tira a linha do tooltip.</x:v>
+        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
       </x:c>
       <x:c r="J1076" s="16" t="str"/>
       <x:c r="K1076" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TooltipLine.js#L18</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L11</x:v>
       </x:c>
     </x:row>
     <x:row r="1077" ht="21.75" customHeight="1">
       <x:c r="A1077" s="16" t="str">
-        <x:v>UsageException</x:v>
+        <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="B1077" s="16" t="str">
-        <x:v>constructor</x:v>
+        <x:v>GetList</x:v>
       </x:c>
       <x:c r="C1077" s="16" t="str">
-        <x:v>Construtor</x:v>
+        <x:v>Instância</x:v>
       </x:c>
       <x:c r="D1077" s="16" t="str">
-        <x:v>constructor(msg, color)</x:v>
+        <x:v>GetList(key)</x:v>
       </x:c>
       <x:c r="E1077" s="16" t="str">
-        <x:v>UsageException</x:v>
+        <x:v>TagCompound</x:v>
       </x:c>
       <x:c r="F1077" s="16" t="str">
         <x:v>Não</x:v>
@@ -37615,23 +37615,254 @@
         <x:v>Declarado</x:v>
       </x:c>
       <x:c r="H1077" s="16" t="str">
-        <x:v>instância</x:v>
+        <x:v>Array.isArray(this[key]) ? this[key] : []</x:v>
       </x:c>
       <x:c r="I1077" s="16" t="str">
-        <x:v>Consulte a implementação na fonte.</x:v>
+        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
       </x:c>
       <x:c r="J1077" s="16" t="str"/>
       <x:c r="K1077" s="16" t="str">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1078" ht="21.75" customHeight="1">
+      <x:c r="A1078" s="16" t="str">
+        <x:v>TagCompound</x:v>
+      </x:c>
+      <x:c r="B1078" s="16" t="str">
+        <x:v>GetString</x:v>
+      </x:c>
+      <x:c r="C1078" s="16" t="str">
+        <x:v>Instância</x:v>
+      </x:c>
+      <x:c r="D1078" s="16" t="str">
+        <x:v>GetString(key)</x:v>
+      </x:c>
+      <x:c r="E1078" s="16" t="str">
+        <x:v>TagCompound</x:v>
+      </x:c>
+      <x:c r="F1078" s="16" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G1078" s="16" t="str">
+        <x:v>Declarado</x:v>
+      </x:c>
+      <x:c r="H1078" s="16" t="str">
+        <x:v>String(this.Get(key, ''))</x:v>
+      </x:c>
+      <x:c r="I1078" s="16" t="str">
+        <x:v>O valor já convertido (falso, 0, '', [] se não há).</x:v>
+      </x:c>
+      <x:c r="J1078" s="16" t="str"/>
+      <x:c r="K1078" s="16" t="str">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1079" ht="21.75" customHeight="1">
+      <x:c r="A1079" s="16" t="str">
+        <x:v>TagCompound</x:v>
+      </x:c>
+      <x:c r="B1079" s="16" t="str">
+        <x:v>Remove</x:v>
+      </x:c>
+      <x:c r="C1079" s="16" t="str">
+        <x:v>Instância</x:v>
+      </x:c>
+      <x:c r="D1079" s="16" t="str">
+        <x:v>Remove(key)</x:v>
+      </x:c>
+      <x:c r="E1079" s="16" t="str">
+        <x:v>TagCompound</x:v>
+      </x:c>
+      <x:c r="F1079" s="16" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G1079" s="16" t="str">
+        <x:v>Declarado</x:v>
+      </x:c>
+      <x:c r="H1079" s="16" t="str">
+        <x:v>Consultar fonte</x:v>
+      </x:c>
+      <x:c r="I1079" s="16" t="str">
+        <x:v>Escrever e apagar.</x:v>
+      </x:c>
+      <x:c r="J1079" s="16" t="str"/>
+      <x:c r="K1079" s="16" t="str">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1080" ht="21.75" customHeight="1">
+      <x:c r="A1080" s="16" t="str">
+        <x:v>TagCompound</x:v>
+      </x:c>
+      <x:c r="B1080" s="16" t="str">
+        <x:v>Set</x:v>
+      </x:c>
+      <x:c r="C1080" s="16" t="str">
+        <x:v>Instância</x:v>
+      </x:c>
+      <x:c r="D1080" s="16" t="str">
+        <x:v>Set(key, value)</x:v>
+      </x:c>
+      <x:c r="E1080" s="16" t="str">
+        <x:v>TagCompound</x:v>
+      </x:c>
+      <x:c r="F1080" s="16" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G1080" s="16" t="str">
+        <x:v>Declarado</x:v>
+      </x:c>
+      <x:c r="H1080" s="16" t="str">
+        <x:v>Consultar fonte</x:v>
+      </x:c>
+      <x:c r="I1080" s="16" t="str">
+        <x:v>Escrever e apagar.</x:v>
+      </x:c>
+      <x:c r="J1080" s="16" t="str"/>
+      <x:c r="K1080" s="16" t="str">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TagCompound.js#L6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1081" ht="21.75" customHeight="1">
+      <x:c r="A1081" s="16" t="str">
+        <x:v>TooltipLine</x:v>
+      </x:c>
+      <x:c r="B1081" s="16" t="str">
+        <x:v>colorTag</x:v>
+      </x:c>
+      <x:c r="C1081" s="16" t="str">
+        <x:v>Estático</x:v>
+      </x:c>
+      <x:c r="D1081" s="16" t="str">
+        <x:v>colorTag(text, color)</x:v>
+      </x:c>
+      <x:c r="E1081" s="16" t="str">
+        <x:v>TooltipLine</x:v>
+      </x:c>
+      <x:c r="F1081" s="16" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G1081" s="16" t="str">
+        <x:v>Declarado</x:v>
+      </x:c>
+      <x:c r="H1081" s="16" t="str">
+        <x:v>'[c/' + TooltipLoader.Hex(color) + ':' + text + ']'</x:v>
+      </x:c>
+      <x:c r="I1081" s="16" t="str">
+        <x:v>'[c/RRGGBB:texto]' para pintar um trecho.</x:v>
+      </x:c>
+      <x:c r="J1081" s="16" t="str"/>
+      <x:c r="K1081" s="16" t="str">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TooltipLine.js#L20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1082" ht="21.75" customHeight="1">
+      <x:c r="A1082" s="16" t="str">
+        <x:v>TooltipLine</x:v>
+      </x:c>
+      <x:c r="B1082" s="16" t="str">
+        <x:v>constructor</x:v>
+      </x:c>
+      <x:c r="C1082" s="16" t="str">
+        <x:v>Construtor</x:v>
+      </x:c>
+      <x:c r="D1082" s="16" t="str">
+        <x:v>constructor(...args)</x:v>
+      </x:c>
+      <x:c r="E1082" s="16" t="str">
+        <x:v>TooltipLine</x:v>
+      </x:c>
+      <x:c r="F1082" s="16" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G1082" s="16" t="str">
+        <x:v>Declarado</x:v>
+      </x:c>
+      <x:c r="H1082" s="16" t="str">
+        <x:v>instância</x:v>
+      </x:c>
+      <x:c r="I1082" s="16" t="str">
+        <x:v>Consulte a implementação na fonte.</x:v>
+      </x:c>
+      <x:c r="J1082" s="16" t="str"/>
+      <x:c r="K1082" s="16" t="str">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TooltipLine.js#L5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1083" ht="21.75" customHeight="1">
+      <x:c r="A1083" s="16" t="str">
+        <x:v>TooltipLine</x:v>
+      </x:c>
+      <x:c r="B1083" s="16" t="str">
+        <x:v>Hide</x:v>
+      </x:c>
+      <x:c r="C1083" s="16" t="str">
+        <x:v>Instância</x:v>
+      </x:c>
+      <x:c r="D1083" s="16" t="str">
+        <x:v>Hide()</x:v>
+      </x:c>
+      <x:c r="E1083" s="16" t="str">
+        <x:v>TooltipLine</x:v>
+      </x:c>
+      <x:c r="F1083" s="16" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G1083" s="16" t="str">
+        <x:v>Declarado</x:v>
+      </x:c>
+      <x:c r="H1083" s="16" t="str">
+        <x:v>Consultar fonte</x:v>
+      </x:c>
+      <x:c r="I1083" s="16" t="str">
+        <x:v>Hide() tira a linha do tooltip.</x:v>
+      </x:c>
+      <x:c r="J1083" s="16" t="str"/>
+      <x:c r="K1083" s="16" t="str">
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/TooltipLine.js#L18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1084" ht="21.75" customHeight="1">
+      <x:c r="A1084" s="16" t="str">
+        <x:v>UsageException</x:v>
+      </x:c>
+      <x:c r="B1084" s="16" t="str">
+        <x:v>constructor</x:v>
+      </x:c>
+      <x:c r="C1084" s="16" t="str">
+        <x:v>Construtor</x:v>
+      </x:c>
+      <x:c r="D1084" s="16" t="str">
+        <x:v>constructor(msg, color)</x:v>
+      </x:c>
+      <x:c r="E1084" s="16" t="str">
+        <x:v>UsageException</x:v>
+      </x:c>
+      <x:c r="F1084" s="16" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G1084" s="16" t="str">
+        <x:v>Declarado</x:v>
+      </x:c>
+      <x:c r="H1084" s="16" t="str">
+        <x:v>instância</x:v>
+      </x:c>
+      <x:c r="I1084" s="16" t="str">
+        <x:v>Consulte a implementação na fonte.</x:v>
+      </x:c>
+      <x:c r="J1084" s="16" t="str"/>
+      <x:c r="K1084" s="16" t="str">
         <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModCommand.js#L45</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G7:G1077">
+  <x:conditionalFormatting sqref="G7:G1084">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Não implementado"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90bd9d48fc047d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra464d0b74e4a4335"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Item.ResearchUnlockCount (Journey mode research), mod items default to 1
</commit_message>
<xml_diff>
--- a/docs/referencia/metodos.xlsx
+++ b/docs/referencia/metodos.xlsx
@@ -22857,7 +22857,7 @@
       </x:c>
       <x:c r="J623" s="16" t="str"/>
       <x:c r="K623" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L416</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L419</x:v>
       </x:c>
     </x:row>
     <x:row r="624" ht="21.75" customHeight="1">
@@ -22960,7 +22960,7 @@
       </x:c>
       <x:c r="J626" s="16" t="str"/>
       <x:c r="K626" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L415</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L418</x:v>
       </x:c>
     </x:row>
     <x:row r="627" ht="21.75" customHeight="1">
@@ -22993,7 +22993,7 @@
       </x:c>
       <x:c r="J627" s="16" t="str"/>
       <x:c r="K627" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L414</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L417</x:v>
       </x:c>
     </x:row>
     <x:row r="628" ht="21.75" customHeight="1">
@@ -23341,7 +23341,7 @@
       </x:c>
       <x:c r="J637" s="16" t="str"/>
       <x:c r="K637" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L413</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L416</x:v>
       </x:c>
     </x:row>
     <x:row r="638" ht="21.75" customHeight="1">
@@ -23374,7 +23374,7 @@
       </x:c>
       <x:c r="J638" s="16" t="str"/>
       <x:c r="K638" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L412</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L415</x:v>
       </x:c>
     </x:row>
     <x:row r="639" ht="21.75" customHeight="1">
@@ -23473,10 +23473,10 @@
         <x:v>Entities.Of(this)</x:v>
       </x:c>
       <x:c r="I641" s="16" t="str">
-        <x:v>game Item</x:v>
+        <x:v>number</x:v>
       </x:c>
       <x:c r="J641" s="16" t="str">
-        <x:v>This instance's item. On the template, undefined.</x:v>
+        <x:v>How many Journey mode asks for to research it (per type). Mod items start at 1; 0 takes the item out of research. Set it in SetStaticDefaults (this.Item.ResearchUnlockCount = 3); it also works on any item, the game's included.</x:v>
       </x:c>
       <x:c r="K641" s="16" t="str">
         <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L13</x:v>

</xml_diff>

<commit_message>
fix: ModBossBar draws through the mobile GUIBossBar.Draw layout, docs updated
</commit_message>
<xml_diff>
--- a/docs/referencia/metodos.xlsx
+++ b/docs/referencia/metodos.xlsx
@@ -18158,7 +18158,7 @@
         <x:v>drawParams: tModLoader's BossBarDrawParams (see GlobalBossBar); false removes the game's drawing.</x:v>
       </x:c>
       <x:c r="J483" s="16" t="str">
-        <x:v>BigProgressBarSystem.Draw → BigProgressBarHelper.DrawFancyBar</x:v>
+        <x:v>BigProgressBarSystem.Draw → GUIBossBar.Draw</x:v>
       </x:c>
       <x:c r="K483" s="16" t="str">
         <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModBossBar.js#L33</x:v>
@@ -18193,7 +18193,7 @@
         <x:v>drawParams: tModLoader's BossBarDrawParams (see GlobalBossBar); false removes the game's drawing.</x:v>
       </x:c>
       <x:c r="J484" s="16" t="str">
-        <x:v>BigProgressBarSystem.Draw → BigProgressBarHelper.DrawFancyBar</x:v>
+        <x:v>BigProgressBarSystem.Draw → GUIBossBar.Draw</x:v>
       </x:c>
       <x:c r="K484" s="16" t="str">
         <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModBossBar.js#L32</x:v>
@@ -22857,7 +22857,7 @@
       </x:c>
       <x:c r="J623" s="16" t="str"/>
       <x:c r="K623" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L419</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L416</x:v>
       </x:c>
     </x:row>
     <x:row r="624" ht="21.75" customHeight="1">
@@ -22960,7 +22960,7 @@
       </x:c>
       <x:c r="J626" s="16" t="str"/>
       <x:c r="K626" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L418</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L415</x:v>
       </x:c>
     </x:row>
     <x:row r="627" ht="21.75" customHeight="1">
@@ -22993,7 +22993,7 @@
       </x:c>
       <x:c r="J627" s="16" t="str"/>
       <x:c r="K627" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L417</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L414</x:v>
       </x:c>
     </x:row>
     <x:row r="628" ht="21.75" customHeight="1">
@@ -23341,7 +23341,7 @@
       </x:c>
       <x:c r="J637" s="16" t="str"/>
       <x:c r="K637" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L416</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L413</x:v>
       </x:c>
     </x:row>
     <x:row r="638" ht="21.75" customHeight="1">
@@ -23374,7 +23374,7 @@
       </x:c>
       <x:c r="J638" s="16" t="str"/>
       <x:c r="K638" s="16" t="str">
-        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L415</x:v>
+        <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L412</x:v>
       </x:c>
     </x:row>
     <x:row r="639" ht="21.75" customHeight="1">
@@ -23473,10 +23473,10 @@
         <x:v>Entities.Of(this)</x:v>
       </x:c>
       <x:c r="I641" s="16" t="str">
-        <x:v>number</x:v>
+        <x:v>game Item</x:v>
       </x:c>
       <x:c r="J641" s="16" t="str">
-        <x:v>How many Journey mode asks for to research it (per type). Mod items start at 1; 0 takes the item out of research. Set it in SetStaticDefaults (this.Item.ResearchUnlockCount = 3); it also works on any item, the game's included.</x:v>
+        <x:v>This instance's item. On the template, undefined.</x:v>
       </x:c>
       <x:c r="K641" s="16" t="str">
         <x:v>https://github.com/JonataOliveiraa/Bunny-Loader/blob/main/app/src/main/cpp/script/js/mod/ModItem.js#L13</x:v>

</xml_diff>